<commit_message>
snapshot 455fc82d1: TAC-B1 deploy: archive files only before safe staged asset replacement
Source-Commit: 455fc82d18031943514c16efa573f621c23da561
</commit_message>
<xml_diff>
--- a/open-world/config/excel/对话.xlsx
+++ b/open-world/config/excel/对话.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R023a2b4eb9564870"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导出" sheetId="2" r:id="R0f63aea055b14921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="3" r:id="R5a156acbd9e247af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="触发" sheetId="4" r:id="R62de5c5a00db4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R10680ebe0dfe41fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导出" sheetId="2" r:id="R1ad86b9505c04446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="对话" sheetId="3" r:id="R9f402def8ee7412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="触发" sheetId="4" r:id="R98bc505a8cd54830"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13539,11 +13539,683 @@
       </x:c>
       <x:c r="F636"/>
     </x:row>
+    <x:row r="637">
+      <x:c r="A637" t="str">
+        <x:v>ow-wind-side-z1-1:accept</x:v>
+      </x:c>
+      <x:c r="B637" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C637" t="str">
+        <x:v>ow-npc-wind-1</x:v>
+      </x:c>
+      <x:c r="D637"/>
+      <x:c r="E637" t="str">
+        <x:v>铃铛没有坏，只是被营地的绳索缠住了。羊群听见它，就知道该往家走。</x:v>
+      </x:c>
+      <x:c r="F637"/>
+    </x:row>
+    <x:row r="638">
+      <x:c r="A638" t="str">
+        <x:v>ow-wind-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B638" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C638" t="str">
+        <x:v>ow-npc-wind-2</x:v>
+      </x:c>
+      <x:c r="D638"/>
+      <x:c r="E638" t="str">
+        <x:v>小艇的木板还能用，先把守着零件的敌人引开。</x:v>
+      </x:c>
+      <x:c r="F638"/>
+    </x:row>
+    <x:row r="639">
+      <x:c r="A639" t="str">
+        <x:v>ow-wind-side-z4-1:accept</x:v>
+      </x:c>
+      <x:c r="B639" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C639" t="str">
+        <x:v>ow-npc-wind-4</x:v>
+      </x:c>
+      <x:c r="D639"/>
+      <x:c r="E639" t="str">
+        <x:v>拾荒者把粮袋留在信标后面，等援兵散去就能带人离开。</x:v>
+      </x:c>
+      <x:c r="F639"/>
+    </x:row>
+    <x:row r="640">
+      <x:c r="A640" t="str">
+        <x:v>ow-wind-side-z6-1:accept</x:v>
+      </x:c>
+      <x:c r="B640" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C640" t="str">
+        <x:v>ow-npc-wind-6</x:v>
+      </x:c>
+      <x:c r="D640"/>
+      <x:c r="E640" t="str">
+        <x:v>信封上的名字还清楚。把货箱打开，就能知道它该寄给谁。</x:v>
+      </x:c>
+      <x:c r="F640"/>
+    </x:row>
+    <x:row r="641">
+      <x:c r="A641" t="str">
+        <x:v>ow-mist-side-z1-1:accept</x:v>
+      </x:c>
+      <x:c r="B641" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C641" t="str">
+        <x:v>ow-npc-mist-1</x:v>
+      </x:c>
+      <x:c r="D641"/>
+      <x:c r="E641" t="str">
+        <x:v>渡船已经偏离邮路，铃声是船夫认得的最后一个路标。</x:v>
+      </x:c>
+      <x:c r="F641"/>
+    </x:row>
+    <x:row r="642">
+      <x:c r="A642" t="str">
+        <x:v>ow-mist-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B642" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C642" t="str">
+        <x:v>ow-npc-mist-2</x:v>
+      </x:c>
+      <x:c r="D642"/>
+      <x:c r="E642" t="str">
+        <x:v>邮包外层湿透了，里面的封蜡还在。别把寄信人的名字弄丢。</x:v>
+      </x:c>
+      <x:c r="F642"/>
+    </x:row>
+    <x:row r="643">
+      <x:c r="A643" t="str">
+        <x:v>ow-mist-side-z5-1:accept</x:v>
+      </x:c>
+      <x:c r="B643" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C643" t="str">
+        <x:v>ow-npc-mist-5</x:v>
+      </x:c>
+      <x:c r="D643"/>
+      <x:c r="E643" t="str">
+        <x:v>难民在信标后等待，守住这里，他们才敢走最后一段路。</x:v>
+      </x:c>
+      <x:c r="F643"/>
+    </x:row>
+    <x:row r="644">
+      <x:c r="A644" t="str">
+        <x:v>ow-mist-side-z6-1:accept</x:v>
+      </x:c>
+      <x:c r="B644" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C644" t="str">
+        <x:v>ow-npc-mist-6</x:v>
+      </x:c>
+      <x:c r="D644"/>
+      <x:c r="E644" t="str">
+        <x:v>工具柄上刻着工匠的名字，和军需货单上的编号对不上。</x:v>
+      </x:c>
+      <x:c r="F644"/>
+    </x:row>
+    <x:row r="645">
+      <x:c r="A645" t="str">
+        <x:v>ow-forge-side-z1-1:accept</x:v>
+      </x:c>
+      <x:c r="B645" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C645" t="str">
+        <x:v>ow-npc-forge-1</x:v>
+      </x:c>
+      <x:c r="D645"/>
+      <x:c r="E645" t="str">
+        <x:v>装载机还在照旧命令运转，后面的工人已经没有退路。</x:v>
+      </x:c>
+      <x:c r="F645"/>
+    </x:row>
+    <x:row r="646">
+      <x:c r="A646" t="str">
+        <x:v>ow-forge-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B646" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C646" t="str">
+        <x:v>ow-npc-forge-2</x:v>
+      </x:c>
+      <x:c r="D646"/>
+      <x:c r="E646" t="str">
+        <x:v>零件不是废料，它们刚好能补上新引擎缺的那一段。</x:v>
+      </x:c>
+      <x:c r="F646"/>
+    </x:row>
+    <x:row r="647">
+      <x:c r="A647" t="str">
+        <x:v>ow-forge-side-z4-1:accept</x:v>
+      </x:c>
+      <x:c r="B647" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C647" t="str">
+        <x:v>ow-npc-forge-4</x:v>
+      </x:c>
+      <x:c r="D647"/>
+      <x:c r="E647" t="str">
+        <x:v>矿道里传来的敲击还没停，先清出一条能让担架通过的路。</x:v>
+      </x:c>
+      <x:c r="F647"/>
+    </x:row>
+    <x:row r="648">
+      <x:c r="A648" t="str">
+        <x:v>ow-forge-side-z6-1:accept</x:v>
+      </x:c>
+      <x:c r="B648" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C648" t="str">
+        <x:v>ow-npc-forge-6</x:v>
+      </x:c>
+      <x:c r="D648"/>
+      <x:c r="E648" t="str">
+        <x:v>工程图上的签名没有被刮掉。技师愿意留下，亲手把错误改回来。</x:v>
+      </x:c>
+      <x:c r="F648"/>
+    </x:row>
+    <x:row r="649">
+      <x:c r="A649" t="str">
+        <x:v>ow-frost-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B649" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C649" t="str">
+        <x:v>ow-npc-frost-2</x:v>
+      </x:c>
+      <x:c r="D649"/>
+      <x:c r="E649" t="str">
+        <x:v>日志的日期停在冰封之前，值更人的名字却一直写到了最后。</x:v>
+      </x:c>
+      <x:c r="F649"/>
+    </x:row>
+    <x:row r="650">
+      <x:c r="A650" t="str">
+        <x:v>ow-frost-side-z3-1:accept</x:v>
+      </x:c>
+      <x:c r="B650" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C650" t="str">
+        <x:v>ow-npc-frost-3</x:v>
+      </x:c>
+      <x:c r="D650"/>
+      <x:c r="E650" t="str">
+        <x:v>两面观测镜还指着同一片海，校准它们就能接上断掉的信号。</x:v>
+      </x:c>
+      <x:c r="F650"/>
+    </x:row>
+    <x:row r="651">
+      <x:c r="A651" t="str">
+        <x:v>ow-frost-side-z4-1:accept</x:v>
+      </x:c>
+      <x:c r="B651" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C651" t="str">
+        <x:v>ow-npc-frost-4</x:v>
+      </x:c>
+      <x:c r="D651"/>
+      <x:c r="E651" t="str">
+        <x:v>侦察兵在冰隙边留了布条，前面的巡守正在向那里靠近。</x:v>
+      </x:c>
+      <x:c r="F651"/>
+    </x:row>
+    <x:row r="652">
+      <x:c r="A652" t="str">
+        <x:v>ow-frost-side-z5-1:accept</x:v>
+      </x:c>
+      <x:c r="B652" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C652" t="str">
+        <x:v>ow-npc-frost-5</x:v>
+      </x:c>
+      <x:c r="D652"/>
+      <x:c r="E652" t="str">
+        <x:v>应答已经迟了很多年，信里的名字仍值得有人认真念出来。</x:v>
+      </x:c>
+      <x:c r="F652"/>
+    </x:row>
+    <x:row r="653">
+      <x:c r="A653" t="str">
+        <x:v>ow-rift-side-z1-1:accept</x:v>
+      </x:c>
+      <x:c r="B653" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C653" t="str">
+        <x:v>ow-npc-rift-1</x:v>
+      </x:c>
+      <x:c r="D653"/>
+      <x:c r="E653" t="str">
+        <x:v>补给箱上的旧货签没被撕掉，里面装的是营地真正需要的东西。</x:v>
+      </x:c>
+      <x:c r="F653"/>
+    </x:row>
+    <x:row r="654">
+      <x:c r="A654" t="str">
+        <x:v>ow-rift-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B654" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C654" t="str">
+        <x:v>ow-npc-rift-2</x:v>
+      </x:c>
+      <x:c r="D654"/>
+      <x:c r="E654" t="str">
+        <x:v>药品清单上有几个孩子的名字，先找齐封存的小箱。</x:v>
+      </x:c>
+      <x:c r="F654"/>
+    </x:row>
+    <x:row r="655">
+      <x:c r="A655" t="str">
+        <x:v>ow-rift-side-z4-1:accept</x:v>
+      </x:c>
+      <x:c r="B655" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C655" t="str">
+        <x:v>ow-npc-rift-4</x:v>
+      </x:c>
+      <x:c r="D655"/>
+      <x:c r="E655" t="str">
+        <x:v>孩子记得母亲留下的记号，守住信标，让她看得见回来的路。</x:v>
+      </x:c>
+      <x:c r="F655"/>
+    </x:row>
+    <x:row r="656">
+      <x:c r="A656" t="str">
+        <x:v>ow-rift-side-z6-1:accept</x:v>
+      </x:c>
+      <x:c r="B656" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C656" t="str">
+        <x:v>ow-npc-rift-6</x:v>
+      </x:c>
+      <x:c r="D656"/>
+      <x:c r="E656" t="str">
+        <x:v>这封信转过好几个哨所。最后一段路，我们替送信的人走完。</x:v>
+      </x:c>
+      <x:c r="F656"/>
+    </x:row>
+    <x:row r="657">
+      <x:c r="A657" t="str">
+        <x:v>ow-dragon-side-z1-1:accept</x:v>
+      </x:c>
+      <x:c r="B657" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C657" t="str">
+        <x:v>ow-npc-dragon-1</x:v>
+      </x:c>
+      <x:c r="D657"/>
+      <x:c r="E657" t="str">
+        <x:v>骨碑上的名字和失物对得上，带回去时别把铭刻磨掉。</x:v>
+      </x:c>
+      <x:c r="F657"/>
+    </x:row>
+    <x:row r="658">
+      <x:c r="A658" t="str">
+        <x:v>ow-dragon-side-z2-1:accept</x:v>
+      </x:c>
+      <x:c r="B658" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C658" t="str">
+        <x:v>ow-npc-dragon-2</x:v>
+      </x:c>
+      <x:c r="D658"/>
+      <x:c r="E658" t="str">
+        <x:v>火盆边还有旧灰。守住这一轮，下一位应答者就能找到这里。</x:v>
+      </x:c>
+      <x:c r="F658"/>
+    </x:row>
+    <x:row r="659">
+      <x:c r="A659" t="str">
+        <x:v>ow-dragon-side-z4-1:accept</x:v>
+      </x:c>
+      <x:c r="B659" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C659" t="str">
+        <x:v>ow-npc-dragon-4</x:v>
+      </x:c>
+      <x:c r="D659"/>
+      <x:c r="E659" t="str">
+        <x:v>看守机的记忆还剩几段，先停下失控的回路，再把它带回去。</x:v>
+      </x:c>
+      <x:c r="F659"/>
+    </x:row>
+    <x:row r="660">
+      <x:c r="A660" t="str">
+        <x:v>ow-dragon-side-z6-1:accept</x:v>
+      </x:c>
+      <x:c r="B660" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C660" t="str">
+        <x:v>ow-npc-dragon-6</x:v>
+      </x:c>
+      <x:c r="D660"/>
+      <x:c r="E660" t="str">
+        <x:v>米洛在航图边留了一处空白，这一箱记录正好能补上。</x:v>
+      </x:c>
+      <x:c r="F660"/>
+    </x:row>
+    <x:row r="661">
+      <x:c r="A661" t="str">
+        <x:v>hub-return:wind-story-1</x:v>
+      </x:c>
+      <x:c r="B661" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C661" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D661"/>
+      <x:c r="E661" t="str">
+        <x:v>船员都回来了，刻片也收好了。</x:v>
+      </x:c>
+      <x:c r="F661"/>
+    </x:row>
+    <x:row r="662">
+      <x:c r="A662" t="str">
+        <x:v>hub-return:wind-story-2</x:v>
+      </x:c>
+      <x:c r="B662" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C662" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D662"/>
+      <x:c r="E662" t="str">
+        <x:v>船台暂时稳住了，大家终于能喘口气。</x:v>
+      </x:c>
+      <x:c r="F662"/>
+    </x:row>
+    <x:row r="663">
+      <x:c r="A663" t="str">
+        <x:v>hub-return:wind-story-3</x:v>
+      </x:c>
+      <x:c r="B663" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C663" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D663"/>
+      <x:c r="E663" t="str">
+        <x:v>两条旧路都记进航图了。</x:v>
+      </x:c>
+      <x:c r="F663"/>
+    </x:row>
+    <x:row r="664">
+      <x:c r="A664" t="str">
+        <x:v>hub-return:mist-story-1</x:v>
+      </x:c>
+      <x:c r="B664" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C664" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D664"/>
+      <x:c r="E664" t="str">
+        <x:v>货单与封条已经收好，下一次再核对来路。</x:v>
+      </x:c>
+      <x:c r="F664"/>
+    </x:row>
+    <x:row r="665">
+      <x:c r="A665" t="str">
+        <x:v>hub-return:mist-story-2</x:v>
+      </x:c>
+      <x:c r="B665" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C665" t="str">
+        <x:v>ss-npc-qingmang</x:v>
+      </x:c>
+      <x:c r="D665"/>
+      <x:c r="E665" t="str">
+        <x:v>青芒已经平安回港，邮包也有了下落。</x:v>
+      </x:c>
+      <x:c r="F665"/>
+    </x:row>
+    <x:row r="666">
+      <x:c r="A666" t="str">
+        <x:v>hub-return:mist-story-3</x:v>
+      </x:c>
+      <x:c r="B666" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C666" t="str">
+        <x:v>ss-npc-qingmang</x:v>
+      </x:c>
+      <x:c r="D666"/>
+      <x:c r="E666" t="str">
+        <x:v>军需队的路线已经记下，回港整理装备。</x:v>
+      </x:c>
+      <x:c r="F666"/>
+    </x:row>
+    <x:row r="667">
+      <x:c r="A667" t="str">
+        <x:v>hub-return:forge-story-1</x:v>
+      </x:c>
+      <x:c r="B667" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C667" t="str">
+        <x:v>ss-npc-tongling</x:v>
+      </x:c>
+      <x:c r="D667"/>
+      <x:c r="E667" t="str">
+        <x:v>冷却阀恢复运转，铜铃收好了输能记录。</x:v>
+      </x:c>
+      <x:c r="F667"/>
+    </x:row>
+    <x:row r="668">
+      <x:c r="A668" t="str">
+        <x:v>hub-return:forge-story-2</x:v>
+      </x:c>
+      <x:c r="B668" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C668" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D668"/>
+      <x:c r="E668" t="str">
+        <x:v>控制台夺回来了，工坊的人有了退路。</x:v>
+      </x:c>
+      <x:c r="F668"/>
+    </x:row>
+    <x:row r="669">
+      <x:c r="A669" t="str">
+        <x:v>hub-return:forge-story-3</x:v>
+      </x:c>
+      <x:c r="B669" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C669" t="str">
+        <x:v>ss-npc-tongling</x:v>
+      </x:c>
+      <x:c r="D669"/>
+      <x:c r="E669" t="str">
+        <x:v>岛心稳住了，新引擎的材料也够了。</x:v>
+      </x:c>
+      <x:c r="F669"/>
+    </x:row>
+    <x:row r="670">
+      <x:c r="A670" t="str">
+        <x:v>hub-return:frost-story-1</x:v>
+      </x:c>
+      <x:c r="B670" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C670" t="str">
+        <x:v>ss-npc-xuemi</x:v>
+      </x:c>
+      <x:c r="D670"/>
+      <x:c r="E670" t="str">
+        <x:v>冻舰的记录带回来了，旧日期仍要仔细核对。</x:v>
+      </x:c>
+      <x:c r="F670"/>
+    </x:row>
+    <x:row r="671">
+      <x:c r="A671" t="str">
+        <x:v>hub-return:frost-story-2</x:v>
+      </x:c>
+      <x:c r="B671" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C671" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D671"/>
+      <x:c r="E671" t="str">
+        <x:v>舰桥通道已经打通，雪弥在港口等你。</x:v>
+      </x:c>
+      <x:c r="F671"/>
+    </x:row>
+    <x:row r="672">
+      <x:c r="A672" t="str">
+        <x:v>hub-return:frost-story-3</x:v>
+      </x:c>
+      <x:c r="B672" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C672" t="str">
+        <x:v>ss-npc-jinyu</x:v>
+      </x:c>
+      <x:c r="D672"/>
+      <x:c r="E672" t="str">
+        <x:v>星图拼好了，航约上的名字一个也没漏。</x:v>
+      </x:c>
+      <x:c r="F672"/>
+    </x:row>
+    <x:row r="673">
+      <x:c r="A673" t="str">
+        <x:v>hub-return:rift-story-1</x:v>
+      </x:c>
+      <x:c r="B673" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C673" t="str">
+        <x:v>ss-npc-mijia</x:v>
+      </x:c>
+      <x:c r="D673"/>
+      <x:c r="E673" t="str">
+        <x:v>证词收齐了，营地里的平民有了退路。</x:v>
+      </x:c>
+      <x:c r="F673"/>
+    </x:row>
+    <x:row r="674">
+      <x:c r="A674" t="str">
+        <x:v>hub-return:rift-story-2</x:v>
+      </x:c>
+      <x:c r="B674" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C674" t="str">
+        <x:v>ss-npc-mijia</x:v>
+      </x:c>
+      <x:c r="D674"/>
+      <x:c r="E674" t="str">
+        <x:v>前哨的守卫退下去了，补给可以运进来。</x:v>
+      </x:c>
+      <x:c r="F674"/>
+    </x:row>
+    <x:row r="675">
+      <x:c r="A675" t="str">
+        <x:v>hub-return:rift-story-3</x:v>
+      </x:c>
+      <x:c r="B675" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C675" t="str">
+        <x:v>ss-npc-mijia</x:v>
+      </x:c>
+      <x:c r="D675"/>
+      <x:c r="E675" t="str">
+        <x:v>供能已经断开，撤离装置仍在运转。</x:v>
+      </x:c>
+      <x:c r="F675"/>
+    </x:row>
+    <x:row r="676">
+      <x:c r="A676" t="str">
+        <x:v>hub-return:dragon-story-1</x:v>
+      </x:c>
+      <x:c r="B676" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C676" t="str">
+        <x:v>ss-npc-jinyu</x:v>
+      </x:c>
+      <x:c r="D676"/>
+      <x:c r="E676" t="str">
+        <x:v>会盟记录带回港口，六岛的应答终于齐了。</x:v>
+      </x:c>
+      <x:c r="F676"/>
+    </x:row>
+    <x:row r="677">
+      <x:c r="A677" t="str">
+        <x:v>hub-return:dragon-story-2</x:v>
+      </x:c>
+      <x:c r="B677" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C677" t="str">
+        <x:v>ss-npc-milo</x:v>
+      </x:c>
+      <x:c r="D677"/>
+      <x:c r="E677" t="str">
+        <x:v>中枢入口打通了，旧航网的声音越来越清楚。</x:v>
+      </x:c>
+      <x:c r="F677"/>
+    </x:row>
+    <x:row r="678">
+      <x:c r="A678" t="str">
+        <x:v>hub-return:dragon-story-3</x:v>
+      </x:c>
+      <x:c r="B678" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C678" t="str">
+        <x:v>ss-npc-jinyu</x:v>
+      </x:c>
+      <x:c r="D678"/>
+      <x:c r="E678" t="str">
+        <x:v>三个航网节点都稳住了，大家准备迎接最后一战。</x:v>
+      </x:c>
+      <x:c r="F678"/>
+    </x:row>
     <x:row r="693" s="6" customFormat="1" ht="32" customHeight="1"/>
     <x:row r="694" s="6" customFormat="1" ht="32" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c527c2875c49cf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b13a4a5915a49f5"/>
 </x:worksheet>
 </file>
 
@@ -13884,6 +14556,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff75533e18874d6e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde78f983bd5a433b"/>
 </x:worksheet>
 </file>
</xml_diff>